<commit_message>
CSV MATCHER (name and dates) UntestedNoData
</commit_message>
<xml_diff>
--- a/local/sheet-updated-from-pdf.xlsx
+++ b/local/sheet-updated-from-pdf.xlsx
@@ -289,16 +289,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1">
-        <v>46121.416666666664</v>
+        <v>46115.458333333336</v>
       </c>
       <c r="B1">
-        <v>-93.08</v>
+        <v>-25.58</v>
       </c>
       <c r="C1" t="str">
-        <v>Superloop Limited BRISBANE</v>
+        <v>ALDI STORES WEST FOOTSCRA AUS</v>
       </c>
       <c r="D1" t="str">
-        <v/>
+        <v>t</v>
       </c>
       <c r="F1" t="str">
         <v>AT A GLANCE</v>
@@ -321,16 +321,16 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <v>46120.416666666664</v>
+        <v>46116.458333333336</v>
       </c>
       <c r="B2">
-        <v>-5.04</v>
+        <v>-9.9</v>
       </c>
       <c r="C2" t="str">
-        <v>COLES 7664 MARIBYRNONG</v>
+        <v>KC CHA PTY LTD. CARLTON</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>n</v>
       </c>
       <c r="F2" s="2">
         <f>SUMIF(D:D, "t", B:B)+Q3+Q4+N3+N2</f>
@@ -370,16 +370,16 @@
     </row>
     <row r="3">
       <c r="A3" s="1">
-        <v>46120.416666666664</v>
+        <v>46117.416666666664</v>
       </c>
       <c r="B3">
-        <v>-22.37</v>
+        <v>-7.9</v>
       </c>
       <c r="C3" t="str">
-        <v>HARVEST MEATS GLEN WAVERLEY AUS</v>
+        <v>Krispy Kreme Highpoint Maribyrnong</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>macq</v>
       </c>
       <c r="F3" s="2">
         <f>SUMIF(D:D, "n", B:B)+R3+R4+O3+O2</f>
@@ -415,13 +415,13 @@
     </row>
     <row r="4">
       <c r="A4" s="1">
-        <v>46120.416666666664</v>
+        <v>46115.458333333336</v>
       </c>
       <c r="B4">
-        <v>-4.2</v>
+        <v>-42.8</v>
       </c>
       <c r="C4" t="str">
-        <v>SMP*Nhu Lan Bakery Fo8 Footscray</v>
+        <v>COLES Footscray</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -447,10 +447,10 @@
         <v>46120.416666666664</v>
       </c>
       <c r="B5">
-        <v>-70.84</v>
+        <v>-89.5</v>
       </c>
       <c r="C5" t="str">
-        <v>VICROADS ONLINE PAYM KEW</v>
+        <v>COLES Footscray</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -464,18 +464,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1">
-        <v>46120.416666666664</v>
-      </c>
-      <c r="B6">
-        <v>-467.58</v>
-      </c>
-      <c r="C6" t="str">
-        <v>VICROADS ONLINE PAYM KEW</v>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
       <c r="F6" s="2">
         <f>SUMIF(D:D, "t", B:B)+Q3</f>
         <v>-1517.14</v>
@@ -485,18 +473,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1">
-        <v>46120.416666666664</v>
-      </c>
-      <c r="B7">
-        <v>-90.31</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Optus Billing MacquariePark AUS</v>
-      </c>
-      <c r="D7" t="str">
-        <v/>
-      </c>
       <c r="F7" s="2">
         <f>SUMIF(D:D, "n", B:B)+R3</f>
         <v>-1597.51</v>
@@ -506,18 +482,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1">
-        <v>46120.416666666664</v>
-      </c>
-      <c r="B8">
-        <v>-22.93</v>
-      </c>
-      <c r="C8" t="str">
-        <v>FOODLE ASIAN GROCERY A MARIBYRNONG</v>
-      </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
       <c r="F8" s="2">
         <f>SUMIF(D:D, "macq", B:B)+S3</f>
         <v>-483.27</v>
@@ -527,41 +491,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1">
-        <v>46119.416666666664</v>
-      </c>
-      <c r="B9">
-        <v>-2.77</v>
-      </c>
-      <c r="C9" t="str">
-        <v>SMARTPLAN CHARGE - COSTCO WHOLESALE AUST</v>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
       <c r="F9" t="str">
         <v>Macq' Balance</v>
       </c>
       <c r="G9" s="2">
-        <v>4356.07</v>
+        <v>0</v>
       </c>
       <c r="H9" t="str">
         <v>&lt;-- Enter CC total. If green, good. If red, bad.</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1">
-        <v>46119.416666666664</v>
-      </c>
-      <c r="B10">
-        <v>-38.45</v>
-      </c>
-      <c r="C10" t="str">
-        <v>McDonalds 950055 SUNSHINE</v>
-      </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
       <c r="F10" s="2">
         <v>-800</v>
       </c>
@@ -577,18 +517,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1">
-        <v>46119.416666666664</v>
-      </c>
-      <c r="B11">
-        <v>-20.2</v>
-      </c>
-      <c r="C11" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
       <c r="F11" t="str">
         <v>Macquerie Excess</v>
       </c>
@@ -600,18 +528,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1">
-        <v>46118.416666666664</v>
-      </c>
-      <c r="B12">
-        <v>-19.1</v>
-      </c>
-      <c r="C12" t="str">
-        <v>McDonalds 950055 SUNSHINE</v>
-      </c>
-      <c r="D12" t="str">
-        <v/>
-      </c>
       <c r="F12" s="2">
         <f>SUM(F10-F4)*-1</f>
         <v>316.73</v>
@@ -635,18 +551,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1">
-        <v>46118.416666666664</v>
-      </c>
-      <c r="B13">
-        <v>-13.1</v>
-      </c>
-      <c r="C13" t="str">
-        <v>BUNNINGS 408000 HIGHPOINT CIT AUS</v>
-      </c>
-      <c r="D13" t="str">
-        <v/>
-      </c>
       <c r="J13" s="2">
         <v>858.4549999999999</v>
       </c>
@@ -663,18 +567,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1">
-        <v>46118.416666666664</v>
-      </c>
-      <c r="B14">
-        <v>-98</v>
-      </c>
-      <c r="C14" t="str">
-        <v>gu health rewards G7 CAMBERWELL</v>
-      </c>
-      <c r="D14" t="str">
-        <v/>
-      </c>
       <c r="G14" s="3" t="str">
         <v>TOTAL</v>
       </c>
@@ -694,18 +586,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1">
-        <v>46118.416666666664</v>
-      </c>
-      <c r="B15">
-        <v>-98.47</v>
-      </c>
-      <c r="C15" t="str">
-        <v>SQ *KARE West Melbourn AUS</v>
-      </c>
-      <c r="D15" t="str">
-        <v/>
-      </c>
       <c r="F15" t="str">
         <v>Tony:</v>
       </c>
@@ -725,18 +605,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1">
-        <v>46118.416666666664</v>
-      </c>
-      <c r="B16">
-        <v>-40.22</v>
-      </c>
-      <c r="C16" t="str">
-        <v>CHEMIST WAREHOUSE MAIDSTONE</v>
-      </c>
-      <c r="D16" t="str">
-        <v/>
-      </c>
       <c r="F16" t="str">
         <v>Nugs:</v>
       </c>
@@ -750,18 +618,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1">
-        <v>46118.416666666664</v>
-      </c>
-      <c r="B17">
-        <v>-15.8</v>
-      </c>
-      <c r="C17" t="str">
-        <v>COLES 7795 BRAYBROOK</v>
-      </c>
-      <c r="D17" t="str">
-        <v/>
-      </c>
       <c r="F17" t="str">
         <v>Macq:</v>
       </c>
@@ -775,18 +631,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1">
-        <v>46117.416666666664</v>
-      </c>
-      <c r="B18">
-        <v>-14</v>
-      </c>
-      <c r="C18" t="str">
-        <v>OFFICEWORKS 0305 MARIBYRNONG</v>
-      </c>
-      <c r="D18" t="str">
-        <v/>
-      </c>
       <c r="F18" t="str">
         <v>Macqbill:</v>
       </c>
@@ -796,18 +640,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1">
-        <v>46117.416666666664</v>
-      </c>
-      <c r="B19">
-        <v>-29.71</v>
-      </c>
-      <c r="C19" t="str">
-        <v>COLES 7691 BRAYBROOK</v>
-      </c>
-      <c r="D19" t="str">
-        <v/>
-      </c>
       <c r="G19" s="2">
         <f>SUM(G15:G18)</f>
         <v>-4077.610317</v>
@@ -817,35 +649,11 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1">
-        <v>46117.416666666664</v>
-      </c>
-      <c r="B20">
-        <v>-47.96</v>
-      </c>
-      <c r="C20" t="str">
-        <v>PETER ALEXANDER MARIBYRNONG</v>
-      </c>
-      <c r="D20" t="str">
-        <v/>
-      </c>
       <c r="J20" t="str">
         <v>COMMON TRANSACTIONS</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1">
-        <v>46117.416666666664</v>
-      </c>
-      <c r="B21">
-        <v>-54.35</v>
-      </c>
-      <c r="C21" t="str">
-        <v>PET CIRCLE 61438333720</v>
-      </c>
-      <c r="D21" t="str">
-        <v/>
-      </c>
       <c r="J21" t="str">
         <v>Paypal</v>
       </c>
@@ -854,18 +662,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1">
-        <v>46116.458333333336</v>
-      </c>
-      <c r="B22">
-        <v>-22.77</v>
-      </c>
-      <c r="C22" t="str">
-        <v>BABA RICH CATERING PT Melbourne</v>
-      </c>
-      <c r="D22" t="str">
-        <v/>
-      </c>
       <c r="F22" t="str">
         <v>Status</v>
       </c>
@@ -884,18 +680,6 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1">
-        <v>46116.458333333336</v>
-      </c>
-      <c r="B23">
-        <v>-16.44</v>
-      </c>
-      <c r="C23" t="str">
-        <v>ANTHROPIC SAN FRANCISCO USA</v>
-      </c>
-      <c r="D23" t="str">
-        <v/>
-      </c>
       <c r="F23" t="str">
         <f>IF(I23=TRUE,"PAID","NOT PAID")</f>
         <v>PAID</v>
@@ -922,18 +706,6 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1">
-        <v>46116.458333333336</v>
-      </c>
-      <c r="B24">
-        <v>-22.22</v>
-      </c>
-      <c r="C24" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D24" t="str">
-        <v/>
-      </c>
       <c r="F24" t="str">
         <f>IF(I24=TRUE,"PAID","NOT PAID")</f>
         <v>PAID</v>
@@ -960,18 +732,6 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1">
-        <v>46116.458333333336</v>
-      </c>
-      <c r="B25">
-        <v>-218.02</v>
-      </c>
-      <c r="C25" t="str">
-        <v>PETBARN 0285953333</v>
-      </c>
-      <c r="D25" t="str">
-        <v/>
-      </c>
       <c r="F25" t="str">
         <f>IF(I25=TRUE,"PAID","NOT PAID")</f>
         <v>PAID</v>
@@ -998,18 +758,6 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1">
-        <v>46115.458333333336</v>
-      </c>
-      <c r="B26">
-        <v>-9.24</v>
-      </c>
-      <c r="C26" t="str">
-        <v>CROWN ASIAN ELIZABETH Melbourne</v>
-      </c>
-      <c r="D26" t="str">
-        <v/>
-      </c>
       <c r="F26" t="str">
         <f>IF(I26=TRUE,"PAID","NOT PAID")</f>
         <v>PAID</v>
@@ -1036,18 +784,6 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1">
-        <v>46115.458333333336</v>
-      </c>
-      <c r="B27">
-        <v>-36.73</v>
-      </c>
-      <c r="C27" t="str">
-        <v>Molly Tea Melbourne</v>
-      </c>
-      <c r="D27" t="str">
-        <v/>
-      </c>
       <c r="F27" s="2">
         <f>SUM(F12*0.333333)</f>
         <v>105.5765611</v>
@@ -1068,18 +804,6 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1">
-        <v>46115.458333333336</v>
-      </c>
-      <c r="B28">
-        <v>-84.85</v>
-      </c>
-      <c r="C28" t="str">
-        <v>SQ *LE BAJO MILKBAR North Melbour AUS</v>
-      </c>
-      <c r="D28" t="str">
-        <v/>
-      </c>
       <c r="G28" t="str">
         <v>At a Glance</v>
       </c>
@@ -1095,18 +819,6 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1">
-        <v>46115.458333333336</v>
-      </c>
-      <c r="B29">
-        <v>-16.44</v>
-      </c>
-      <c r="C29" t="str">
-        <v>ANTHROPIC SAN FRANCISCO USA</v>
-      </c>
-      <c r="D29" t="str">
-        <v/>
-      </c>
       <c r="F29" t="str">
         <v>Grocery</v>
       </c>
@@ -1126,18 +838,6 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1">
-        <v>46114.458333333336</v>
-      </c>
-      <c r="B30">
-        <v>-6.47</v>
-      </c>
-      <c r="C30" t="str">
-        <v>EasyPark PRAHRAN</v>
-      </c>
-      <c r="D30" t="str">
-        <v/>
-      </c>
       <c r="F30" t="str">
         <v>Fast Food</v>
       </c>
@@ -1161,18 +861,6 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1">
-        <v>46114.458333333336</v>
-      </c>
-      <c r="B31">
-        <v>-169.49</v>
-      </c>
-      <c r="C31" t="str">
-        <v>RED ENERGY CREMORNE</v>
-      </c>
-      <c r="D31" t="str">
-        <v/>
-      </c>
       <c r="F31" t="str">
         <v>Resturant/Cafe</v>
       </c>
@@ -1193,18 +881,6 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1">
-        <v>46114.458333333336</v>
-      </c>
-      <c r="B32">
-        <v>-188.58</v>
-      </c>
-      <c r="C32" t="str">
-        <v>Uniqlo Emporium Melbourne</v>
-      </c>
-      <c r="D32" t="str">
-        <v/>
-      </c>
       <c r="G32" s="2">
         <f>SUM(G17:G18)</f>
         <v>-1279.69</v>
@@ -1221,18 +897,6 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1">
-        <v>46114.458333333336</v>
-      </c>
-      <c r="B33">
-        <v>-20.2</v>
-      </c>
-      <c r="C33" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D33" t="str">
-        <v/>
-      </c>
       <c r="G33" s="2">
         <f>SUM(G15:G18)</f>
         <v>-4077.610317</v>
@@ -1249,18 +913,6 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1">
-        <v>46113.458333333336</v>
-      </c>
-      <c r="B34">
-        <v>-21.03</v>
-      </c>
-      <c r="C34" t="str">
-        <v>COLES 7795 BRAYBROOK</v>
-      </c>
-      <c r="D34" t="str">
-        <v/>
-      </c>
       <c r="M34">
         <f>SUM(M32-M33)</f>
         <v>3364.78</v>
@@ -1274,18 +926,6 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1">
-        <v>46113.458333333336</v>
-      </c>
-      <c r="B35">
-        <v>-100</v>
-      </c>
-      <c r="C35" t="str">
-        <v>Bras N Things Kew</v>
-      </c>
-      <c r="D35" t="str">
-        <v/>
-      </c>
       <c r="F35" t="str">
         <v>Tony:</v>
       </c>
@@ -1305,18 +945,6 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1">
-        <v>46113.458333333336</v>
-      </c>
-      <c r="B36">
-        <v>-8.39</v>
-      </c>
-      <c r="C36" t="str">
-        <v>CENTRAL WEST ASIAN FOO BRAYBROOK</v>
-      </c>
-      <c r="D36" t="str">
-        <v/>
-      </c>
       <c r="F36" t="str">
         <v>Nugs:</v>
       </c>
@@ -1337,18 +965,6 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1">
-        <v>46112.458333333336</v>
-      </c>
-      <c r="B37">
-        <v>-36.85</v>
-      </c>
-      <c r="C37" t="str">
-        <v>KFC Sunshine Sunshine</v>
-      </c>
-      <c r="D37" t="str">
-        <v/>
-      </c>
       <c r="N37">
         <v>2400</v>
       </c>
@@ -1365,18 +981,6 @@
       </c>
     </row>
     <row r="38" xml:space="preserve">
-      <c r="A38" s="1">
-        <v>46112.458333333336</v>
-      </c>
-      <c r="B38">
-        <v>-145</v>
-      </c>
-      <c r="C38" t="str">
-        <v>Mecca Brands Pty Ltd Richmond</v>
-      </c>
-      <c r="D38" t="str">
-        <v/>
-      </c>
       <c r="E38" t="str">
         <v>350 uniql;o</v>
       </c>
@@ -1401,18 +1005,6 @@
       </c>
     </row>
     <row r="39" xml:space="preserve">
-      <c r="A39" s="1">
-        <v>46112.458333333336</v>
-      </c>
-      <c r="B39">
-        <v>-20.2</v>
-      </c>
-      <c r="C39" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D39" t="str">
-        <v/>
-      </c>
       <c r="E39" t="str">
         <v>25 w retail</v>
       </c>
@@ -1444,18 +1036,6 @@
       </c>
     </row>
     <row r="40" xml:space="preserve">
-      <c r="A40" s="1">
-        <v>46111.458333333336</v>
-      </c>
-      <c r="B40">
-        <v>-73.2</v>
-      </c>
-      <c r="C40" t="str">
-        <v>COLES 7691 BRAYBROOK</v>
-      </c>
-      <c r="D40" t="str">
-        <v/>
-      </c>
       <c r="E40" t="str">
         <v>100 spotlight</v>
       </c>
@@ -1483,18 +1063,6 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1">
-        <v>46111.458333333336</v>
-      </c>
-      <c r="B41">
-        <v>-3.98</v>
-      </c>
-      <c r="C41" t="str">
-        <v>COSTCO WHOLESALE AUSTR ARDEER</v>
-      </c>
-      <c r="D41" t="str">
-        <v/>
-      </c>
       <c r="F41" s="2">
         <f>SUM(G17,G18)</f>
         <v>-1279.69</v>
@@ -1516,18 +1084,6 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1">
-        <v>46111.458333333336</v>
-      </c>
-      <c r="B42">
-        <v>-277.32</v>
-      </c>
-      <c r="C42" t="str">
-        <v>COSTCO WHOLESALE AUSTR ARDEER</v>
-      </c>
-      <c r="D42" t="str">
-        <v/>
-      </c>
       <c r="I42">
         <v>1104.66</v>
       </c>
@@ -1547,18 +1103,6 @@
       </c>
     </row>
     <row r="43" xml:space="preserve">
-      <c r="A43" s="1">
-        <v>46111.458333333336</v>
-      </c>
-      <c r="B43">
-        <v>-8.99</v>
-      </c>
-      <c r="C43" t="str">
-        <v>COSTCO WHOLESALE AUSTR ARDEER</v>
-      </c>
-      <c r="D43" t="str">
-        <v/>
-      </c>
       <c r="I43">
         <v>476.42</v>
       </c>
@@ -1582,18 +1126,6 @@
       </c>
     </row>
     <row r="44" xml:space="preserve">
-      <c r="A44" s="1">
-        <v>46111.458333333336</v>
-      </c>
-      <c r="B44">
-        <v>-24.33</v>
-      </c>
-      <c r="C44" t="str">
-        <v>PAYPAL *GOOGLE GRAVITY 4029357733</v>
-      </c>
-      <c r="D44" t="str">
-        <v/>
-      </c>
       <c r="I44">
         <f>SUM(I41:I43)</f>
         <v>3818.31</v>
@@ -1618,18 +1150,6 @@
       </c>
     </row>
     <row r="45" xml:space="preserve">
-      <c r="A45" s="1">
-        <v>46110.458333333336</v>
-      </c>
-      <c r="B45">
-        <v>-14.72</v>
-      </c>
-      <c r="C45" t="str">
-        <v>LS W COSMETICS AUBURN</v>
-      </c>
-      <c r="D45" t="str">
-        <v/>
-      </c>
       <c r="E45">
         <f>SUM(B12,B18,B24,B28,B31,B34,B43,B50,B57,B69,B75,B81,B88,B102,B104)</f>
         <v>-604.17</v>
@@ -1669,18 +1189,6 @@
       </c>
     </row>
     <row r="46" xml:space="preserve">
-      <c r="A46" s="1">
-        <v>46110.458333333336</v>
-      </c>
-      <c r="B46">
-        <v>-81.6</v>
-      </c>
-      <c r="C46" t="str">
-        <v>COLES 7795 BRAYBROOK</v>
-      </c>
-      <c r="D46" t="str">
-        <v/>
-      </c>
       <c r="F46">
         <f>SUM(F45/4)</f>
         <v>493.6425</v>
@@ -1715,18 +1223,6 @@
       </c>
     </row>
     <row r="47" xml:space="preserve">
-      <c r="A47" s="1">
-        <v>46110.458333333336</v>
-      </c>
-      <c r="B47">
-        <v>-32.2</v>
-      </c>
-      <c r="C47" t="str">
-        <v>McDonalds 950055 SUNSHINE</v>
-      </c>
-      <c r="D47" t="str">
-        <v/>
-      </c>
       <c r="F47">
         <f xml:space="preserve">SUM(F46*0.33) </f>
         <v>162.902025</v>
@@ -1751,18 +1247,6 @@
       </c>
     </row>
     <row r="48" xml:space="preserve">
-      <c r="A48" s="1">
-        <v>46110.458333333336</v>
-      </c>
-      <c r="B48">
-        <v>-22.22</v>
-      </c>
-      <c r="C48" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D48" t="str">
-        <v/>
-      </c>
       <c r="F48">
         <f>SUM(F46*0.66)</f>
         <v>325.80405</v>
@@ -1787,18 +1271,6 @@
       </c>
     </row>
     <row r="49" xml:space="preserve">
-      <c r="A49" s="1">
-        <v>46109.458333333336</v>
-      </c>
-      <c r="B49">
-        <v>-6.47</v>
-      </c>
-      <c r="C49" t="str">
-        <v>EasyPark PRAHRAN</v>
-      </c>
-      <c r="D49" t="str">
-        <v/>
-      </c>
       <c r="F49" t="str">
         <v>NEXT CREDIT CARD</v>
       </c>
@@ -1830,18 +1302,6 @@
       </c>
     </row>
     <row r="50" xml:space="preserve">
-      <c r="A50" s="1">
-        <v>46109.458333333336</v>
-      </c>
-      <c r="B50">
-        <v>-22.22</v>
-      </c>
-      <c r="C50" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D50" t="str">
-        <v/>
-      </c>
       <c r="I50">
         <f>SUM(561.83+800)</f>
         <v>1361.83</v>
@@ -1863,18 +1323,6 @@
       </c>
     </row>
     <row r="51" xml:space="preserve">
-      <c r="A51" s="1">
-        <v>46108.458333333336</v>
-      </c>
-      <c r="B51">
-        <v>-85.39</v>
-      </c>
-      <c r="C51" t="str">
-        <v>RED ENERGY CREMORNE</v>
-      </c>
-      <c r="D51" t="str">
-        <v/>
-      </c>
       <c r="F51">
         <v>2432.6396736</v>
       </c>
@@ -1903,18 +1351,6 @@
       </c>
     </row>
     <row r="52" xml:space="preserve">
-      <c r="A52" s="1">
-        <v>46108.458333333336</v>
-      </c>
-      <c r="B52">
-        <v>-5.5</v>
-      </c>
-      <c r="C52" t="str">
-        <v>READING ROOM CAFE QPS FOOTSCRAY</v>
-      </c>
-      <c r="D52" t="str">
-        <v/>
-      </c>
       <c r="F52">
         <v>214.0198368</v>
       </c>
@@ -1939,18 +1375,6 @@
       </c>
     </row>
     <row r="53" xml:space="preserve">
-      <c r="A53" s="1">
-        <v>46108.458333333336</v>
-      </c>
-      <c r="B53">
-        <v>-138.92</v>
-      </c>
-      <c r="C53" t="str">
-        <v>MR BROOKS PTY LTD BRAYBROOK</v>
-      </c>
-      <c r="D53" t="str">
-        <v/>
-      </c>
       <c r="N53" t="str">
         <v>Migrant Coffee</v>
       </c>
@@ -1968,18 +1392,6 @@
       </c>
     </row>
     <row r="54" xml:space="preserve">
-      <c r="A54" s="1">
-        <v>46107.458333333336</v>
-      </c>
-      <c r="B54">
-        <v>-6.56</v>
-      </c>
-      <c r="C54" t="str">
-        <v>EasyPark PRAHRAN</v>
-      </c>
-      <c r="D54" t="str">
-        <v/>
-      </c>
       <c r="F54" t="str">
         <v>OWING TO MACQBILL REMAINING</v>
       </c>
@@ -2003,18 +1415,6 @@
       </c>
     </row>
     <row r="55" xml:space="preserve">
-      <c r="A55" s="1">
-        <v>46107.458333333336</v>
-      </c>
-      <c r="B55">
-        <v>-14.94</v>
-      </c>
-      <c r="C55" t="str">
-        <v>LITTLESPARROW B0526 MELBOURNE</v>
-      </c>
-      <c r="D55" t="str">
-        <v/>
-      </c>
       <c r="F55">
         <v>325.80405</v>
       </c>
@@ -2041,18 +1441,6 @@
       </c>
     </row>
     <row r="56" xml:space="preserve">
-      <c r="A56" s="1">
-        <v>46107.458333333336</v>
-      </c>
-      <c r="B56">
-        <v>-8.09</v>
-      </c>
-      <c r="C56" t="str">
-        <v>Google Ragnarok Origi SINGAPORE</v>
-      </c>
-      <c r="D56" t="str">
-        <v/>
-      </c>
       <c r="F56" t="str">
         <v>PAID in SEPT</v>
       </c>
@@ -2077,18 +1465,6 @@
       </c>
     </row>
     <row r="57" xml:space="preserve">
-      <c r="A57" s="1">
-        <v>46107.458333333336</v>
-      </c>
-      <c r="B57">
-        <v>-20.2</v>
-      </c>
-      <c r="C57" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D57" t="str">
-        <v/>
-      </c>
       <c r="F57">
         <f>SUM(B3,B4,B7,B11,B23,B27,B28,B33,B38,B42,B48,B49,B50,B56,B61,B69,B70,B71,B73,B76,B82,B85,B86,B94)</f>
         <v>-874.8</v>
@@ -2116,18 +1492,6 @@
       </c>
     </row>
     <row r="58" xml:space="preserve">
-      <c r="A58" s="1">
-        <v>46106.458333333336</v>
-      </c>
-      <c r="B58">
-        <v>-51.09</v>
-      </c>
-      <c r="C58" t="str">
-        <v>Bonds Outlet Sunshine Sunshine</v>
-      </c>
-      <c r="D58" t="str">
-        <v/>
-      </c>
       <c r="F58">
         <f>SUM(B9,B10,B13,B14,B17,B20,B26,B36,B43,B44,B47,B51,B55,B72,B74,B81,B83,B90,B99)</f>
         <v>-1164.33</v>
@@ -2152,18 +1516,6 @@
       </c>
     </row>
     <row r="59" xml:space="preserve">
-      <c r="A59" s="1">
-        <v>46106.458333333336</v>
-      </c>
-      <c r="B59">
-        <v>-46.49</v>
-      </c>
-      <c r="C59" t="str">
-        <v>WOOLWORTHS 3186 SUNSHINE</v>
-      </c>
-      <c r="D59" t="str">
-        <v/>
-      </c>
       <c r="I59">
         <f>SUM(I57:I58)</f>
         <v>561.83</v>
@@ -2189,18 +1541,6 @@
       </c>
     </row>
     <row r="60" xml:space="preserve">
-      <c r="A60" s="1">
-        <v>46106.458333333336</v>
-      </c>
-      <c r="B60">
-        <v>-8.15</v>
-      </c>
-      <c r="C60" t="str">
-        <v>ANTHROPIC SAN FRANCISCO USA</v>
-      </c>
-      <c r="D60" t="str">
-        <v/>
-      </c>
       <c r="I60">
         <v>800</v>
       </c>
@@ -2221,18 +1561,6 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1">
-        <v>46105.458333333336</v>
-      </c>
-      <c r="B61">
-        <v>-6.56</v>
-      </c>
-      <c r="C61" t="str">
-        <v>EasyPark PRAHRAN</v>
-      </c>
-      <c r="D61" t="str">
-        <v/>
-      </c>
       <c r="F61" s="2">
         <v>3985.81261566</v>
       </c>
@@ -2252,18 +1580,6 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1">
-        <v>46105.458333333336</v>
-      </c>
-      <c r="B62">
-        <v>-20.2</v>
-      </c>
-      <c r="C62" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D62" t="str">
-        <v/>
-      </c>
       <c r="F62">
         <v>3652.5</v>
       </c>
@@ -2284,18 +1600,6 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1">
-        <v>46104.458333333336</v>
-      </c>
-      <c r="B63">
-        <v>-15.45</v>
-      </c>
-      <c r="C63" t="str">
-        <v>SUNO INC. CAMBRIDGE</v>
-      </c>
-      <c r="D63" t="str">
-        <v/>
-      </c>
       <c r="E63" t="str">
         <v>INVESTIGATE</v>
       </c>
@@ -2316,18 +1620,6 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1">
-        <v>46104.458333333336</v>
-      </c>
-      <c r="B64">
-        <v>-31.45</v>
-      </c>
-      <c r="C64" t="str">
-        <v>HJs Highpoint Maribyrnong</v>
-      </c>
-      <c r="D64" t="str">
-        <v/>
-      </c>
       <c r="J64" s="2" t="str">
         <v>Latest Formula 9pm</v>
       </c>
@@ -2340,18 +1632,6 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1">
-        <v>46104.458333333336</v>
-      </c>
-      <c r="B65">
-        <v>-17.48</v>
-      </c>
-      <c r="C65" t="str">
-        <v>DUMPLING ALLEY HP MARIBYRNONG</v>
-      </c>
-      <c r="D65" t="str">
-        <v/>
-      </c>
       <c r="F65">
         <v>325.8</v>
       </c>
@@ -2373,18 +1653,6 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1">
-        <v>46104.458333333336</v>
-      </c>
-      <c r="B66">
-        <v>-37.3</v>
-      </c>
-      <c r="C66" t="str">
-        <v>FOODLE ASIAN GROCERY A MARIBYRNONG</v>
-      </c>
-      <c r="D66" t="str">
-        <v/>
-      </c>
       <c r="I66" s="5" t="str">
         <v>+</v>
       </c>
@@ -2406,18 +1674,6 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1">
-        <v>46104.458333333336</v>
-      </c>
-      <c r="B67">
-        <v>-17.79</v>
-      </c>
-      <c r="C67" t="str">
-        <v>FOODLE ASIAN GROCERY A MARIBYRNONG</v>
-      </c>
-      <c r="D67" t="str">
-        <v/>
-      </c>
       <c r="F67" t="str">
         <v>1.5k (500 downsairs) took 200 for vinnies kid</v>
       </c>
@@ -2442,18 +1698,6 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1">
-        <v>46103.458333333336</v>
-      </c>
-      <c r="B68">
-        <v>-49.15</v>
-      </c>
-      <c r="C68" t="str">
-        <v>SQ *COBB LANE BAKERY Yarraville</v>
-      </c>
-      <c r="D68" t="str">
-        <v/>
-      </c>
       <c r="F68" t="str">
         <v>tony paid vinnies' -200 (2.3)</v>
       </c>
@@ -2475,18 +1719,6 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1">
-        <v>46103.458333333336</v>
-      </c>
-      <c r="B69">
-        <v>-3.2</v>
-      </c>
-      <c r="C69" t="str">
-        <v>COLES 7795 BRAYBROOK</v>
-      </c>
-      <c r="D69" t="str">
-        <v/>
-      </c>
       <c r="F69" t="str">
         <v>AS OF 11/23/2025</v>
       </c>
@@ -2505,18 +1737,6 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B70">
-        <v>-38.93</v>
-      </c>
-      <c r="C70" t="str">
-        <v>NENE CHICKEN SUNSHINE SUNSHINE</v>
-      </c>
-      <c r="D70" t="str">
-        <v/>
-      </c>
       <c r="F70" t="str">
         <v>macqbill owes tony 2.5</v>
       </c>
@@ -2538,18 +1758,6 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B71">
-        <v>-26.83</v>
-      </c>
-      <c r="C71" t="str">
-        <v>SQ *INDUS SPECIALTY CO St Kilda</v>
-      </c>
-      <c r="D71" t="str">
-        <v/>
-      </c>
       <c r="F71" t="str">
         <v>macqbill owes tony 2.3</v>
       </c>
@@ -2568,18 +1776,6 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B72">
-        <v>-15.23</v>
-      </c>
-      <c r="C72" t="str">
-        <v>KOMIKO.APP SAN FRANCISCO USA</v>
-      </c>
-      <c r="D72" t="str">
-        <v/>
-      </c>
       <c r="F72" s="2" t="str">
         <v>Macbill owes tony $1178</v>
       </c>
@@ -2598,18 +1794,6 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B73">
-        <v>-52.99</v>
-      </c>
-      <c r="C73" t="str">
-        <v>SQ *FOOD &amp; WINE EXPO Williamstown AUS</v>
-      </c>
-      <c r="D73" t="str">
-        <v/>
-      </c>
       <c r="F73" s="2" t="str">
         <v>Nugs owe macbill $561</v>
       </c>
@@ -2622,18 +1806,6 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B74">
-        <v>-22.22</v>
-      </c>
-      <c r="C74" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D74" t="str">
-        <v/>
-      </c>
       <c r="Q74">
         <v>-28.55</v>
       </c>
@@ -2643,18 +1815,6 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B75">
-        <v>-37.9</v>
-      </c>
-      <c r="C75" t="str">
-        <v>LS *BellPizza Mount Waverle AUS</v>
-      </c>
-      <c r="D75" t="str">
-        <v/>
-      </c>
       <c r="F75" t="str">
         <v>Nugs owe macbill $311 as of 22/01/2025</v>
       </c>
@@ -2671,18 +1831,6 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B76">
-        <v>-18.89</v>
-      </c>
-      <c r="C76" t="str">
-        <v>PAYPAL *LEMONSQUEEZ 4029357733</v>
-      </c>
-      <c r="D76" t="str">
-        <v/>
-      </c>
       <c r="F76" t="str">
         <v xml:space="preserve">Jan bill &gt; Nugs to add 155.5 to "Japan" </v>
       </c>
@@ -2698,18 +1846,6 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1">
-        <v>46101.458333333336</v>
-      </c>
-      <c r="B77">
-        <v>-44</v>
-      </c>
-      <c r="C77" t="str">
-        <v>POP MART OCEANIA PTY L MELBOURNE</v>
-      </c>
-      <c r="D77" t="str">
-        <v/>
-      </c>
       <c r="F77" t="str">
         <v xml:space="preserve">Feb bill &gt; Nugs to add 155.5 to "Japan" </v>
       </c>
@@ -2725,18 +1861,6 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1">
-        <v>46101.458333333336</v>
-      </c>
-      <c r="B78">
-        <v>-9.6</v>
-      </c>
-      <c r="C78" t="str">
-        <v>WOOLWORTHS 3079 MARIBYRNONG</v>
-      </c>
-      <c r="D78" t="str">
-        <v/>
-      </c>
       <c r="Q78">
         <v>-1.03</v>
       </c>
@@ -2746,18 +1870,6 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1">
-        <v>46101.458333333336</v>
-      </c>
-      <c r="B79">
-        <v>-41.99</v>
-      </c>
-      <c r="C79" t="str">
-        <v>SQ *JASPER HIGHPOINT Maribyrnong</v>
-      </c>
-      <c r="D79" t="str">
-        <v/>
-      </c>
       <c r="Q79">
         <v>-0.49</v>
       </c>
@@ -2767,18 +1879,6 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1">
-        <v>46101.458333333336</v>
-      </c>
-      <c r="B80">
-        <v>-45.27</v>
-      </c>
-      <c r="C80" t="str">
-        <v>DUMPLING PLUS MARIBYRNONG</v>
-      </c>
-      <c r="D80" t="str">
-        <v/>
-      </c>
       <c r="Q80">
         <v>-37.5</v>
       </c>
@@ -2788,18 +1888,6 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1">
-        <v>46101.458333333336</v>
-      </c>
-      <c r="B81">
-        <v>-38</v>
-      </c>
-      <c r="C81" t="str">
-        <v>HARVEY NORMAN AV/IT MARIBYRNONG</v>
-      </c>
-      <c r="D81" t="str">
-        <v/>
-      </c>
       <c r="Q81">
         <v>-16.82</v>
       </c>
@@ -2809,18 +1897,6 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1">
-        <v>46101.458333333336</v>
-      </c>
-      <c r="B82">
-        <v>-30.98</v>
-      </c>
-      <c r="C82" t="str">
-        <v>PLINE PH HIGHPOINT MARIBYRNONG</v>
-      </c>
-      <c r="D82" t="str">
-        <v/>
-      </c>
       <c r="Q82">
         <v>-99.2</v>
       </c>
@@ -2830,18 +1906,6 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1">
-        <v>46100.458333333336</v>
-      </c>
-      <c r="B83">
-        <v>-42.65</v>
-      </c>
-      <c r="C83" t="str">
-        <v>McDonalds 950055 SUNSHINE</v>
-      </c>
-      <c r="D83" t="str">
-        <v/>
-      </c>
       <c r="Q83">
         <v>-66</v>
       </c>
@@ -2850,92 +1914,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="1">
-        <v>46098.458333333336</v>
-      </c>
-      <c r="B84">
-        <v>-631.43</v>
-      </c>
-      <c r="C84" t="str">
-        <v>GWW SUNBURY</v>
-      </c>
-      <c r="D84" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="1">
-        <v>46097.458333333336</v>
-      </c>
-      <c r="B85">
-        <v>-17.8</v>
-      </c>
-      <c r="C85" t="str">
-        <v>COLES 7795 BRAYBROOK</v>
-      </c>
-      <c r="D85" t="str">
-        <v/>
-      </c>
-    </row>
     <row r="86">
-      <c r="A86" s="1">
-        <v>46097.458333333336</v>
-      </c>
-      <c r="B86">
-        <v>-4.99</v>
-      </c>
-      <c r="C86" t="str">
-        <v>CENTRAL WEST ASIAN FOO BRAYBROOK</v>
-      </c>
-      <c r="D86" t="str">
-        <v/>
-      </c>
       <c r="F86">
         <v>1090</v>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="1">
-        <v>46097.458333333336</v>
-      </c>
-      <c r="B87">
-        <v>-21.14</v>
-      </c>
-      <c r="C87" t="str">
-        <v>KFL SUPERMARKET BRAYBR BRAYBROOK</v>
-      </c>
-      <c r="D87" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="1">
-        <v>46097.458333333336</v>
-      </c>
-      <c r="B88">
-        <v>-65</v>
-      </c>
-      <c r="C88" t="str">
-        <v>Superloop Limited BRISBANE</v>
-      </c>
-      <c r="D88" t="str">
-        <v/>
-      </c>
-    </row>
     <row r="89">
-      <c r="A89" s="1">
-        <v>46097.458333333336</v>
-      </c>
-      <c r="B89">
-        <v>-7.92</v>
-      </c>
-      <c r="C89" t="str">
-        <v>S &amp; S PRODUCE PTY LT BRAYBROOK</v>
-      </c>
-      <c r="D89" t="str">
-        <v/>
-      </c>
       <c r="G89">
         <v>399.96</v>
       </c>
@@ -2951,18 +1935,6 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1">
-        <v>46097.458333333336</v>
-      </c>
-      <c r="B90">
-        <v>-8.61</v>
-      </c>
-      <c r="C90" t="str">
-        <v>ALDI STORES WEST FOOTSCRA AUS</v>
-      </c>
-      <c r="D90" t="str">
-        <v/>
-      </c>
       <c r="G90">
         <v>199.98</v>
       </c>
@@ -2974,120 +1946,12 @@
         <v>66.66</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="1">
-        <v>46096.458333333336</v>
-      </c>
-      <c r="B91">
-        <v>-39.9</v>
-      </c>
-      <c r="C91" t="str">
-        <v>COLES 7795 BRAYBROOK</v>
-      </c>
-      <c r="D91" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="1">
-        <v>46096.458333333336</v>
-      </c>
-      <c r="B92">
-        <v>-22.43</v>
-      </c>
-      <c r="C92" t="str">
-        <v>Pacific D.lit Taylors Hill AUS</v>
-      </c>
-      <c r="D92" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="1">
-        <v>46096.458333333336</v>
-      </c>
-      <c r="B93">
-        <v>-131.25</v>
-      </c>
-      <c r="C93" t="str">
-        <v>Supre Sydney</v>
-      </c>
-      <c r="D93" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="1">
-        <v>46096.458333333336</v>
-      </c>
-      <c r="B94">
-        <v>-49.95</v>
-      </c>
-      <c r="C94" t="str">
-        <v>UPDOC--L.UPDOC.CO/CP SURRY HILLS</v>
-      </c>
-      <c r="D94" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="1">
-        <v>46096.458333333336</v>
-      </c>
-      <c r="B95">
-        <v>-25.58</v>
-      </c>
-      <c r="C95" t="str">
-        <v>ALDI STORES WEST FOOTSCRA AUS</v>
-      </c>
-      <c r="D95" t="str">
-        <v>t</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="1">
-        <v>46095.458333333336</v>
-      </c>
-      <c r="B96">
-        <v>-9.9</v>
-      </c>
-      <c r="C96" t="str">
-        <v>KC CHA PTY LTD. CARLTON</v>
-      </c>
-      <c r="D96" t="str">
-        <v>n</v>
-      </c>
-    </row>
     <row r="97">
-      <c r="A97" s="1">
-        <v>46095.458333333336</v>
-      </c>
-      <c r="B97">
-        <v>-7.9</v>
-      </c>
-      <c r="C97" t="str">
-        <v>Krispy Kreme Highpoint Maribyrnong</v>
-      </c>
-      <c r="D97" t="str">
-        <v>macq</v>
-      </c>
       <c r="G97" s="2">
         <v>6253.47</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1">
-        <v>46094.458333333336</v>
-      </c>
-      <c r="B98">
-        <v>-19.81</v>
-      </c>
-      <c r="C98" t="str">
-        <v>SQ *OLD MAN PHO EMPORI Melbourne</v>
-      </c>
-      <c r="D98" t="str">
-        <v>t</v>
-      </c>
       <c r="G98" t="str">
         <v/>
       </c>
@@ -3097,18 +1961,6 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1">
-        <v>46094.458333333336</v>
-      </c>
-      <c r="B99">
-        <v>-9.38</v>
-      </c>
-      <c r="C99" t="str">
-        <v>CWH MELBOURNE CENTRAL MELBOURNE</v>
-      </c>
-      <c r="D99" t="str">
-        <v/>
-      </c>
       <c r="G99" s="3" t="str">
         <v>Havies Distributed</v>
       </c>
@@ -3118,38 +1970,12 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1">
-        <v>46093.458333333336</v>
-      </c>
-      <c r="B100">
-        <v>-47.45</v>
-      </c>
-      <c r="C100" t="str">
-        <v>COLES 7664 MARIBYRNONG</v>
-      </c>
-      <c r="D100" t="str">
-        <v/>
-      </c>
       <c r="G100" s="2">
         <v>371.18499999999983</v>
       </c>
       <c r="H100">
         <f>SUM(H98:H99)</f>
         <v>12540</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="1">
-        <v>46093.458333333336</v>
-      </c>
-      <c r="B101">
-        <v>-21.19</v>
-      </c>
-      <c r="C101" t="str">
-        <v>FOODLE ASIAN GROCERY A MARIBYRNONG</v>
-      </c>
-      <c r="D101" t="str">
-        <v/>
       </c>
     </row>
     <row r="102">
@@ -3298,16 +2124,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1">
-        <v>46121.416666666664</v>
+        <v>46115.458333333336</v>
       </c>
       <c r="B1">
-        <v>-93.08</v>
+        <v>-25.58</v>
       </c>
       <c r="C1" t="str">
-        <v>Superloop Limited BRISBANE</v>
+        <v>ALDI STORES WEST FOOTSCRA AUS</v>
       </c>
       <c r="D1" t="str">
-        <v/>
+        <v>t</v>
       </c>
       <c r="F1" t="str">
         <v>AT A GLANCE</v>
@@ -3330,16 +2156,16 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <v>46120.416666666664</v>
+        <v>46116.458333333336</v>
       </c>
       <c r="B2">
-        <v>-5.04</v>
+        <v>-9.9</v>
       </c>
       <c r="C2" t="str">
-        <v>COLES 7664 MARIBYRNONG</v>
+        <v>KC CHA PTY LTD. CARLTON</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>n</v>
       </c>
       <c r="F2" s="2">
         <f>SUMIF(D:D, "t", B:B)+Q3+Q4+N3+N2</f>
@@ -3379,16 +2205,16 @@
     </row>
     <row r="3">
       <c r="A3" s="1">
-        <v>46120.416666666664</v>
+        <v>46117.416666666664</v>
       </c>
       <c r="B3">
-        <v>-22.37</v>
+        <v>-7.9</v>
       </c>
       <c r="C3" t="str">
-        <v>HARVEST MEATS GLEN WAVERLEY AUS</v>
+        <v>Krispy Kreme Highpoint Maribyrnong</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>macq</v>
       </c>
       <c r="F3" s="2">
         <f>SUMIF(D:D, "n", B:B)+R3+R4+O3+O2</f>
@@ -3424,13 +2250,13 @@
     </row>
     <row r="4">
       <c r="A4" s="1">
-        <v>46120.416666666664</v>
+        <v>46115.458333333336</v>
       </c>
       <c r="B4">
-        <v>-4.2</v>
+        <v>-42.8</v>
       </c>
       <c r="C4" t="str">
-        <v>SMP*Nhu Lan Bakery Fo8 Footscray</v>
+        <v>COLES Footscray</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -3456,10 +2282,10 @@
         <v>46120.416666666664</v>
       </c>
       <c r="B5">
-        <v>-70.84</v>
+        <v>-89.5</v>
       </c>
       <c r="C5" t="str">
-        <v>VICROADS ONLINE PAYM KEW</v>
+        <v>COLES Footscray</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -3473,18 +2299,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1">
-        <v>46120.416666666664</v>
-      </c>
-      <c r="B6">
-        <v>-467.58</v>
-      </c>
-      <c r="C6" t="str">
-        <v>VICROADS ONLINE PAYM KEW</v>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
       <c r="F6" s="2">
         <f>SUMIF(D:D, "t", B:B)+Q3</f>
         <v>-1517.14</v>
@@ -3494,18 +2308,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1">
-        <v>46120.416666666664</v>
-      </c>
-      <c r="B7">
-        <v>-90.31</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Optus Billing MacquariePark AUS</v>
-      </c>
-      <c r="D7" t="str">
-        <v/>
-      </c>
       <c r="F7" s="2">
         <f>SUMIF(D:D, "n", B:B)+R3</f>
         <v>-1597.51</v>
@@ -3515,18 +2317,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1">
-        <v>46120.416666666664</v>
-      </c>
-      <c r="B8">
-        <v>-22.93</v>
-      </c>
-      <c r="C8" t="str">
-        <v>FOODLE ASIAN GROCERY A MARIBYRNONG</v>
-      </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
       <c r="F8" s="2">
         <f>SUMIF(D:D, "macq", B:B)+S3</f>
         <v>-483.27</v>
@@ -3536,41 +2326,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1">
-        <v>46119.416666666664</v>
-      </c>
-      <c r="B9">
-        <v>-2.77</v>
-      </c>
-      <c r="C9" t="str">
-        <v>SMARTPLAN CHARGE - COSTCO WHOLESALE AUST</v>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
       <c r="F9" t="str">
         <v>Macq' Balance</v>
       </c>
       <c r="G9" s="2">
-        <v>4356.07</v>
+        <v>0</v>
       </c>
       <c r="H9" t="str">
         <v>&lt;-- Enter CC total. If green, good. If red, bad.</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1">
-        <v>46119.416666666664</v>
-      </c>
-      <c r="B10">
-        <v>-38.45</v>
-      </c>
-      <c r="C10" t="str">
-        <v>McDonalds 950055 SUNSHINE</v>
-      </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
       <c r="F10" s="2">
         <v>-800</v>
       </c>
@@ -3586,18 +2352,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1">
-        <v>46119.416666666664</v>
-      </c>
-      <c r="B11">
-        <v>-20.2</v>
-      </c>
-      <c r="C11" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
       <c r="F11" t="str">
         <v>Macquerie Excess</v>
       </c>
@@ -3609,18 +2363,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1">
-        <v>46118.416666666664</v>
-      </c>
-      <c r="B12">
-        <v>-19.1</v>
-      </c>
-      <c r="C12" t="str">
-        <v>McDonalds 950055 SUNSHINE</v>
-      </c>
-      <c r="D12" t="str">
-        <v/>
-      </c>
       <c r="F12" s="2">
         <f>SUM(F10-F4)*-1</f>
         <v>316.73</v>
@@ -3644,18 +2386,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1">
-        <v>46118.416666666664</v>
-      </c>
-      <c r="B13">
-        <v>-13.1</v>
-      </c>
-      <c r="C13" t="str">
-        <v>BUNNINGS 408000 HIGHPOINT CIT AUS</v>
-      </c>
-      <c r="D13" t="str">
-        <v/>
-      </c>
       <c r="J13" s="2">
         <v>858.4549999999999</v>
       </c>
@@ -3672,18 +2402,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1">
-        <v>46118.416666666664</v>
-      </c>
-      <c r="B14">
-        <v>-98</v>
-      </c>
-      <c r="C14" t="str">
-        <v>gu health rewards G7 CAMBERWELL</v>
-      </c>
-      <c r="D14" t="str">
-        <v/>
-      </c>
       <c r="G14" s="3" t="str">
         <v>TOTAL</v>
       </c>
@@ -3703,18 +2421,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1">
-        <v>46118.416666666664</v>
-      </c>
-      <c r="B15">
-        <v>-98.47</v>
-      </c>
-      <c r="C15" t="str">
-        <v>SQ *KARE West Melbourn AUS</v>
-      </c>
-      <c r="D15" t="str">
-        <v/>
-      </c>
       <c r="F15" t="str">
         <v>Tony:</v>
       </c>
@@ -3734,18 +2440,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1">
-        <v>46118.416666666664</v>
-      </c>
-      <c r="B16">
-        <v>-40.22</v>
-      </c>
-      <c r="C16" t="str">
-        <v>CHEMIST WAREHOUSE MAIDSTONE</v>
-      </c>
-      <c r="D16" t="str">
-        <v/>
-      </c>
       <c r="F16" t="str">
         <v>Nugs:</v>
       </c>
@@ -3759,18 +2453,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1">
-        <v>46118.416666666664</v>
-      </c>
-      <c r="B17">
-        <v>-15.8</v>
-      </c>
-      <c r="C17" t="str">
-        <v>COLES 7795 BRAYBROOK</v>
-      </c>
-      <c r="D17" t="str">
-        <v/>
-      </c>
       <c r="F17" t="str">
         <v>Macq:</v>
       </c>
@@ -3784,18 +2466,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1">
-        <v>46117.416666666664</v>
-      </c>
-      <c r="B18">
-        <v>-14</v>
-      </c>
-      <c r="C18" t="str">
-        <v>OFFICEWORKS 0305 MARIBYRNONG</v>
-      </c>
-      <c r="D18" t="str">
-        <v/>
-      </c>
       <c r="F18" t="str">
         <v>Macqbill:</v>
       </c>
@@ -3805,18 +2475,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1">
-        <v>46117.416666666664</v>
-      </c>
-      <c r="B19">
-        <v>-29.71</v>
-      </c>
-      <c r="C19" t="str">
-        <v>COLES 7691 BRAYBROOK</v>
-      </c>
-      <c r="D19" t="str">
-        <v/>
-      </c>
       <c r="G19" s="2">
         <f>SUM(G15:G18)</f>
         <v>-4077.610317</v>
@@ -3826,35 +2484,11 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1">
-        <v>46117.416666666664</v>
-      </c>
-      <c r="B20">
-        <v>-47.96</v>
-      </c>
-      <c r="C20" t="str">
-        <v>PETER ALEXANDER MARIBYRNONG</v>
-      </c>
-      <c r="D20" t="str">
-        <v/>
-      </c>
       <c r="J20" t="str">
         <v>COMMON TRANSACTIONS</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1">
-        <v>46117.416666666664</v>
-      </c>
-      <c r="B21">
-        <v>-54.35</v>
-      </c>
-      <c r="C21" t="str">
-        <v>PET CIRCLE 61438333720</v>
-      </c>
-      <c r="D21" t="str">
-        <v/>
-      </c>
       <c r="J21" t="str">
         <v>Paypal</v>
       </c>
@@ -3863,18 +2497,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1">
-        <v>46116.458333333336</v>
-      </c>
-      <c r="B22">
-        <v>-22.77</v>
-      </c>
-      <c r="C22" t="str">
-        <v>BABA RICH CATERING PT Melbourne</v>
-      </c>
-      <c r="D22" t="str">
-        <v/>
-      </c>
       <c r="F22" t="str">
         <v>Status</v>
       </c>
@@ -3893,18 +2515,6 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1">
-        <v>46116.458333333336</v>
-      </c>
-      <c r="B23">
-        <v>-16.44</v>
-      </c>
-      <c r="C23" t="str">
-        <v>ANTHROPIC SAN FRANCISCO USA</v>
-      </c>
-      <c r="D23" t="str">
-        <v/>
-      </c>
       <c r="F23" t="str">
         <f>IF(I23=TRUE,"PAID","NOT PAID")</f>
         <v>PAID</v>
@@ -3931,18 +2541,6 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1">
-        <v>46116.458333333336</v>
-      </c>
-      <c r="B24">
-        <v>-22.22</v>
-      </c>
-      <c r="C24" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D24" t="str">
-        <v/>
-      </c>
       <c r="F24" t="str">
         <f>IF(I24=TRUE,"PAID","NOT PAID")</f>
         <v>PAID</v>
@@ -3969,18 +2567,6 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1">
-        <v>46116.458333333336</v>
-      </c>
-      <c r="B25">
-        <v>-218.02</v>
-      </c>
-      <c r="C25" t="str">
-        <v>PETBARN 0285953333</v>
-      </c>
-      <c r="D25" t="str">
-        <v/>
-      </c>
       <c r="F25" t="str">
         <f>IF(I25=TRUE,"PAID","NOT PAID")</f>
         <v>PAID</v>
@@ -4007,18 +2593,6 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1">
-        <v>46115.458333333336</v>
-      </c>
-      <c r="B26">
-        <v>-9.24</v>
-      </c>
-      <c r="C26" t="str">
-        <v>CROWN ASIAN ELIZABETH Melbourne</v>
-      </c>
-      <c r="D26" t="str">
-        <v/>
-      </c>
       <c r="F26" t="str">
         <f>IF(I26=TRUE,"PAID","NOT PAID")</f>
         <v>PAID</v>
@@ -4045,18 +2619,6 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1">
-        <v>46115.458333333336</v>
-      </c>
-      <c r="B27">
-        <v>-36.73</v>
-      </c>
-      <c r="C27" t="str">
-        <v>Molly Tea Melbourne</v>
-      </c>
-      <c r="D27" t="str">
-        <v/>
-      </c>
       <c r="F27" s="2">
         <f>SUM(F12*0.333333)</f>
         <v>105.5765611</v>
@@ -4077,18 +2639,6 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1">
-        <v>46115.458333333336</v>
-      </c>
-      <c r="B28">
-        <v>-84.85</v>
-      </c>
-      <c r="C28" t="str">
-        <v>SQ *LE BAJO MILKBAR North Melbour AUS</v>
-      </c>
-      <c r="D28" t="str">
-        <v/>
-      </c>
       <c r="G28" t="str">
         <v>At a Glance</v>
       </c>
@@ -4104,18 +2654,6 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1">
-        <v>46115.458333333336</v>
-      </c>
-      <c r="B29">
-        <v>-16.44</v>
-      </c>
-      <c r="C29" t="str">
-        <v>ANTHROPIC SAN FRANCISCO USA</v>
-      </c>
-      <c r="D29" t="str">
-        <v/>
-      </c>
       <c r="F29" t="str">
         <v>Grocery</v>
       </c>
@@ -4135,18 +2673,6 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1">
-        <v>46114.458333333336</v>
-      </c>
-      <c r="B30">
-        <v>-6.47</v>
-      </c>
-      <c r="C30" t="str">
-        <v>EasyPark PRAHRAN</v>
-      </c>
-      <c r="D30" t="str">
-        <v/>
-      </c>
       <c r="F30" t="str">
         <v>Fast Food</v>
       </c>
@@ -4170,18 +2696,6 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1">
-        <v>46114.458333333336</v>
-      </c>
-      <c r="B31">
-        <v>-169.49</v>
-      </c>
-      <c r="C31" t="str">
-        <v>RED ENERGY CREMORNE</v>
-      </c>
-      <c r="D31" t="str">
-        <v/>
-      </c>
       <c r="F31" t="str">
         <v>Resturant/Cafe</v>
       </c>
@@ -4202,18 +2716,6 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1">
-        <v>46114.458333333336</v>
-      </c>
-      <c r="B32">
-        <v>-188.58</v>
-      </c>
-      <c r="C32" t="str">
-        <v>Uniqlo Emporium Melbourne</v>
-      </c>
-      <c r="D32" t="str">
-        <v/>
-      </c>
       <c r="G32" s="2">
         <f>SUM(G17:G18)</f>
         <v>-1279.69</v>
@@ -4230,18 +2732,6 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1">
-        <v>46114.458333333336</v>
-      </c>
-      <c r="B33">
-        <v>-20.2</v>
-      </c>
-      <c r="C33" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D33" t="str">
-        <v/>
-      </c>
       <c r="G33" s="2">
         <f>SUM(G15:G18)</f>
         <v>-4077.610317</v>
@@ -4258,18 +2748,6 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1">
-        <v>46113.458333333336</v>
-      </c>
-      <c r="B34">
-        <v>-21.03</v>
-      </c>
-      <c r="C34" t="str">
-        <v>COLES 7795 BRAYBROOK</v>
-      </c>
-      <c r="D34" t="str">
-        <v/>
-      </c>
       <c r="M34">
         <f>SUM(M32-M33)</f>
         <v>3364.78</v>
@@ -4283,18 +2761,6 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1">
-        <v>46113.458333333336</v>
-      </c>
-      <c r="B35">
-        <v>-100</v>
-      </c>
-      <c r="C35" t="str">
-        <v>Bras N Things Kew</v>
-      </c>
-      <c r="D35" t="str">
-        <v/>
-      </c>
       <c r="F35" t="str">
         <v>Tony:</v>
       </c>
@@ -4314,18 +2780,6 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1">
-        <v>46113.458333333336</v>
-      </c>
-      <c r="B36">
-        <v>-8.39</v>
-      </c>
-      <c r="C36" t="str">
-        <v>CENTRAL WEST ASIAN FOO BRAYBROOK</v>
-      </c>
-      <c r="D36" t="str">
-        <v/>
-      </c>
       <c r="F36" t="str">
         <v>Nugs:</v>
       </c>
@@ -4346,18 +2800,6 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1">
-        <v>46112.458333333336</v>
-      </c>
-      <c r="B37">
-        <v>-36.85</v>
-      </c>
-      <c r="C37" t="str">
-        <v>KFC Sunshine Sunshine</v>
-      </c>
-      <c r="D37" t="str">
-        <v/>
-      </c>
       <c r="N37">
         <v>2400</v>
       </c>
@@ -4374,18 +2816,6 @@
       </c>
     </row>
     <row r="38" xml:space="preserve">
-      <c r="A38" s="1">
-        <v>46112.458333333336</v>
-      </c>
-      <c r="B38">
-        <v>-145</v>
-      </c>
-      <c r="C38" t="str">
-        <v>Mecca Brands Pty Ltd Richmond</v>
-      </c>
-      <c r="D38" t="str">
-        <v/>
-      </c>
       <c r="E38" t="str">
         <v>350 uniql;o</v>
       </c>
@@ -4410,18 +2840,6 @@
       </c>
     </row>
     <row r="39" xml:space="preserve">
-      <c r="A39" s="1">
-        <v>46112.458333333336</v>
-      </c>
-      <c r="B39">
-        <v>-20.2</v>
-      </c>
-      <c r="C39" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D39" t="str">
-        <v/>
-      </c>
       <c r="E39" t="str">
         <v>25 w retail</v>
       </c>
@@ -4453,18 +2871,6 @@
       </c>
     </row>
     <row r="40" xml:space="preserve">
-      <c r="A40" s="1">
-        <v>46111.458333333336</v>
-      </c>
-      <c r="B40">
-        <v>-73.2</v>
-      </c>
-      <c r="C40" t="str">
-        <v>COLES 7691 BRAYBROOK</v>
-      </c>
-      <c r="D40" t="str">
-        <v/>
-      </c>
       <c r="E40" t="str">
         <v>100 spotlight</v>
       </c>
@@ -4492,18 +2898,6 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1">
-        <v>46111.458333333336</v>
-      </c>
-      <c r="B41">
-        <v>-3.98</v>
-      </c>
-      <c r="C41" t="str">
-        <v>COSTCO WHOLESALE AUSTR ARDEER</v>
-      </c>
-      <c r="D41" t="str">
-        <v/>
-      </c>
       <c r="F41" s="2">
         <f>SUM(G17,G18)</f>
         <v>-1279.69</v>
@@ -4525,18 +2919,6 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1">
-        <v>46111.458333333336</v>
-      </c>
-      <c r="B42">
-        <v>-277.32</v>
-      </c>
-      <c r="C42" t="str">
-        <v>COSTCO WHOLESALE AUSTR ARDEER</v>
-      </c>
-      <c r="D42" t="str">
-        <v/>
-      </c>
       <c r="I42">
         <v>1104.66</v>
       </c>
@@ -4556,18 +2938,6 @@
       </c>
     </row>
     <row r="43" xml:space="preserve">
-      <c r="A43" s="1">
-        <v>46111.458333333336</v>
-      </c>
-      <c r="B43">
-        <v>-8.99</v>
-      </c>
-      <c r="C43" t="str">
-        <v>COSTCO WHOLESALE AUSTR ARDEER</v>
-      </c>
-      <c r="D43" t="str">
-        <v/>
-      </c>
       <c r="I43">
         <v>476.42</v>
       </c>
@@ -4591,18 +2961,6 @@
       </c>
     </row>
     <row r="44" xml:space="preserve">
-      <c r="A44" s="1">
-        <v>46111.458333333336</v>
-      </c>
-      <c r="B44">
-        <v>-24.33</v>
-      </c>
-      <c r="C44" t="str">
-        <v>PAYPAL *GOOGLE GRAVITY 4029357733</v>
-      </c>
-      <c r="D44" t="str">
-        <v/>
-      </c>
       <c r="I44">
         <f>SUM(I41:I43)</f>
         <v>3818.31</v>
@@ -4627,18 +2985,6 @@
       </c>
     </row>
     <row r="45" xml:space="preserve">
-      <c r="A45" s="1">
-        <v>46110.458333333336</v>
-      </c>
-      <c r="B45">
-        <v>-14.72</v>
-      </c>
-      <c r="C45" t="str">
-        <v>LS W COSMETICS AUBURN</v>
-      </c>
-      <c r="D45" t="str">
-        <v/>
-      </c>
       <c r="E45">
         <f>SUM(B12,B18,B24,B28,B31,B34,B43,B50,B57,B69,B75,B81,B88,B102,B104)</f>
         <v>-604.17</v>
@@ -4678,18 +3024,6 @@
       </c>
     </row>
     <row r="46" xml:space="preserve">
-      <c r="A46" s="1">
-        <v>46110.458333333336</v>
-      </c>
-      <c r="B46">
-        <v>-81.6</v>
-      </c>
-      <c r="C46" t="str">
-        <v>COLES 7795 BRAYBROOK</v>
-      </c>
-      <c r="D46" t="str">
-        <v/>
-      </c>
       <c r="F46">
         <f>SUM(F45/4)</f>
         <v>493.6425</v>
@@ -4724,18 +3058,6 @@
       </c>
     </row>
     <row r="47" xml:space="preserve">
-      <c r="A47" s="1">
-        <v>46110.458333333336</v>
-      </c>
-      <c r="B47">
-        <v>-32.2</v>
-      </c>
-      <c r="C47" t="str">
-        <v>McDonalds 950055 SUNSHINE</v>
-      </c>
-      <c r="D47" t="str">
-        <v/>
-      </c>
       <c r="F47">
         <f xml:space="preserve">SUM(F46*0.33) </f>
         <v>162.902025</v>
@@ -4760,18 +3082,6 @@
       </c>
     </row>
     <row r="48" xml:space="preserve">
-      <c r="A48" s="1">
-        <v>46110.458333333336</v>
-      </c>
-      <c r="B48">
-        <v>-22.22</v>
-      </c>
-      <c r="C48" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D48" t="str">
-        <v/>
-      </c>
       <c r="F48">
         <f>SUM(F46*0.66)</f>
         <v>325.80405</v>
@@ -4796,18 +3106,6 @@
       </c>
     </row>
     <row r="49" xml:space="preserve">
-      <c r="A49" s="1">
-        <v>46109.458333333336</v>
-      </c>
-      <c r="B49">
-        <v>-6.47</v>
-      </c>
-      <c r="C49" t="str">
-        <v>EasyPark PRAHRAN</v>
-      </c>
-      <c r="D49" t="str">
-        <v/>
-      </c>
       <c r="F49" t="str">
         <v>NEXT CREDIT CARD</v>
       </c>
@@ -4839,18 +3137,6 @@
       </c>
     </row>
     <row r="50" xml:space="preserve">
-      <c r="A50" s="1">
-        <v>46109.458333333336</v>
-      </c>
-      <c r="B50">
-        <v>-22.22</v>
-      </c>
-      <c r="C50" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D50" t="str">
-        <v/>
-      </c>
       <c r="I50">
         <f>SUM(561.83+800)</f>
         <v>1361.83</v>
@@ -4872,18 +3158,6 @@
       </c>
     </row>
     <row r="51" xml:space="preserve">
-      <c r="A51" s="1">
-        <v>46108.458333333336</v>
-      </c>
-      <c r="B51">
-        <v>-85.39</v>
-      </c>
-      <c r="C51" t="str">
-        <v>RED ENERGY CREMORNE</v>
-      </c>
-      <c r="D51" t="str">
-        <v/>
-      </c>
       <c r="F51">
         <v>2432.6396736</v>
       </c>
@@ -4912,18 +3186,6 @@
       </c>
     </row>
     <row r="52" xml:space="preserve">
-      <c r="A52" s="1">
-        <v>46108.458333333336</v>
-      </c>
-      <c r="B52">
-        <v>-5.5</v>
-      </c>
-      <c r="C52" t="str">
-        <v>READING ROOM CAFE QPS FOOTSCRAY</v>
-      </c>
-      <c r="D52" t="str">
-        <v/>
-      </c>
       <c r="F52">
         <v>214.0198368</v>
       </c>
@@ -4948,18 +3210,6 @@
       </c>
     </row>
     <row r="53" xml:space="preserve">
-      <c r="A53" s="1">
-        <v>46108.458333333336</v>
-      </c>
-      <c r="B53">
-        <v>-138.92</v>
-      </c>
-      <c r="C53" t="str">
-        <v>MR BROOKS PTY LTD BRAYBROOK</v>
-      </c>
-      <c r="D53" t="str">
-        <v/>
-      </c>
       <c r="N53" t="str">
         <v>Migrant Coffee</v>
       </c>
@@ -4977,18 +3227,6 @@
       </c>
     </row>
     <row r="54" xml:space="preserve">
-      <c r="A54" s="1">
-        <v>46107.458333333336</v>
-      </c>
-      <c r="B54">
-        <v>-6.56</v>
-      </c>
-      <c r="C54" t="str">
-        <v>EasyPark PRAHRAN</v>
-      </c>
-      <c r="D54" t="str">
-        <v/>
-      </c>
       <c r="F54" t="str">
         <v>OWING TO MACQBILL REMAINING</v>
       </c>
@@ -5012,18 +3250,6 @@
       </c>
     </row>
     <row r="55" xml:space="preserve">
-      <c r="A55" s="1">
-        <v>46107.458333333336</v>
-      </c>
-      <c r="B55">
-        <v>-14.94</v>
-      </c>
-      <c r="C55" t="str">
-        <v>LITTLESPARROW B0526 MELBOURNE</v>
-      </c>
-      <c r="D55" t="str">
-        <v/>
-      </c>
       <c r="F55">
         <v>325.80405</v>
       </c>
@@ -5050,18 +3276,6 @@
       </c>
     </row>
     <row r="56" xml:space="preserve">
-      <c r="A56" s="1">
-        <v>46107.458333333336</v>
-      </c>
-      <c r="B56">
-        <v>-8.09</v>
-      </c>
-      <c r="C56" t="str">
-        <v>Google Ragnarok Origi SINGAPORE</v>
-      </c>
-      <c r="D56" t="str">
-        <v/>
-      </c>
       <c r="F56" t="str">
         <v>PAID in SEPT</v>
       </c>
@@ -5086,18 +3300,6 @@
       </c>
     </row>
     <row r="57" xml:space="preserve">
-      <c r="A57" s="1">
-        <v>46107.458333333336</v>
-      </c>
-      <c r="B57">
-        <v>-20.2</v>
-      </c>
-      <c r="C57" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D57" t="str">
-        <v/>
-      </c>
       <c r="F57">
         <f>SUM(B3,B4,B7,B11,B23,B27,B28,B33,B38,B42,B48,B49,B50,B56,B61,B69,B70,B71,B73,B76,B82,B85,B86,B94)</f>
         <v>-874.8</v>
@@ -5125,18 +3327,6 @@
       </c>
     </row>
     <row r="58" xml:space="preserve">
-      <c r="A58" s="1">
-        <v>46106.458333333336</v>
-      </c>
-      <c r="B58">
-        <v>-51.09</v>
-      </c>
-      <c r="C58" t="str">
-        <v>Bonds Outlet Sunshine Sunshine</v>
-      </c>
-      <c r="D58" t="str">
-        <v/>
-      </c>
       <c r="F58">
         <f>SUM(B9,B10,B13,B14,B17,B20,B26,B36,B43,B44,B47,B51,B55,B72,B74,B81,B83,B90,B99)</f>
         <v>-1164.33</v>
@@ -5161,18 +3351,6 @@
       </c>
     </row>
     <row r="59" xml:space="preserve">
-      <c r="A59" s="1">
-        <v>46106.458333333336</v>
-      </c>
-      <c r="B59">
-        <v>-46.49</v>
-      </c>
-      <c r="C59" t="str">
-        <v>WOOLWORTHS 3186 SUNSHINE</v>
-      </c>
-      <c r="D59" t="str">
-        <v/>
-      </c>
       <c r="I59">
         <f>SUM(I57:I58)</f>
         <v>561.83</v>
@@ -5198,18 +3376,6 @@
       </c>
     </row>
     <row r="60" xml:space="preserve">
-      <c r="A60" s="1">
-        <v>46106.458333333336</v>
-      </c>
-      <c r="B60">
-        <v>-8.15</v>
-      </c>
-      <c r="C60" t="str">
-        <v>ANTHROPIC SAN FRANCISCO USA</v>
-      </c>
-      <c r="D60" t="str">
-        <v/>
-      </c>
       <c r="I60">
         <v>800</v>
       </c>
@@ -5230,18 +3396,6 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1">
-        <v>46105.458333333336</v>
-      </c>
-      <c r="B61">
-        <v>-6.56</v>
-      </c>
-      <c r="C61" t="str">
-        <v>EasyPark PRAHRAN</v>
-      </c>
-      <c r="D61" t="str">
-        <v/>
-      </c>
       <c r="F61" s="2">
         <v>3985.81261566</v>
       </c>
@@ -5261,18 +3415,6 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1">
-        <v>46105.458333333336</v>
-      </c>
-      <c r="B62">
-        <v>-20.2</v>
-      </c>
-      <c r="C62" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D62" t="str">
-        <v/>
-      </c>
       <c r="F62">
         <v>3652.5</v>
       </c>
@@ -5293,18 +3435,6 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1">
-        <v>46104.458333333336</v>
-      </c>
-      <c r="B63">
-        <v>-15.45</v>
-      </c>
-      <c r="C63" t="str">
-        <v>SUNO INC. CAMBRIDGE</v>
-      </c>
-      <c r="D63" t="str">
-        <v/>
-      </c>
       <c r="E63" t="str">
         <v>INVESTIGATE</v>
       </c>
@@ -5325,18 +3455,6 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1">
-        <v>46104.458333333336</v>
-      </c>
-      <c r="B64">
-        <v>-31.45</v>
-      </c>
-      <c r="C64" t="str">
-        <v>HJs Highpoint Maribyrnong</v>
-      </c>
-      <c r="D64" t="str">
-        <v/>
-      </c>
       <c r="J64" s="2" t="str">
         <v>Latest Formula 9pm</v>
       </c>
@@ -5349,18 +3467,6 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1">
-        <v>46104.458333333336</v>
-      </c>
-      <c r="B65">
-        <v>-17.48</v>
-      </c>
-      <c r="C65" t="str">
-        <v>DUMPLING ALLEY HP MARIBYRNONG</v>
-      </c>
-      <c r="D65" t="str">
-        <v/>
-      </c>
       <c r="F65">
         <v>325.8</v>
       </c>
@@ -5382,18 +3488,6 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1">
-        <v>46104.458333333336</v>
-      </c>
-      <c r="B66">
-        <v>-37.3</v>
-      </c>
-      <c r="C66" t="str">
-        <v>FOODLE ASIAN GROCERY A MARIBYRNONG</v>
-      </c>
-      <c r="D66" t="str">
-        <v/>
-      </c>
       <c r="I66" s="5" t="str">
         <v>+</v>
       </c>
@@ -5415,18 +3509,6 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1">
-        <v>46104.458333333336</v>
-      </c>
-      <c r="B67">
-        <v>-17.79</v>
-      </c>
-      <c r="C67" t="str">
-        <v>FOODLE ASIAN GROCERY A MARIBYRNONG</v>
-      </c>
-      <c r="D67" t="str">
-        <v/>
-      </c>
       <c r="F67" t="str">
         <v>1.5k (500 downsairs) took 200 for vinnies kid</v>
       </c>
@@ -5451,18 +3533,6 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1">
-        <v>46103.458333333336</v>
-      </c>
-      <c r="B68">
-        <v>-49.15</v>
-      </c>
-      <c r="C68" t="str">
-        <v>SQ *COBB LANE BAKERY Yarraville</v>
-      </c>
-      <c r="D68" t="str">
-        <v/>
-      </c>
       <c r="F68" t="str">
         <v>tony paid vinnies' -200 (2.3)</v>
       </c>
@@ -5484,18 +3554,6 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1">
-        <v>46103.458333333336</v>
-      </c>
-      <c r="B69">
-        <v>-3.2</v>
-      </c>
-      <c r="C69" t="str">
-        <v>COLES 7795 BRAYBROOK</v>
-      </c>
-      <c r="D69" t="str">
-        <v/>
-      </c>
       <c r="F69" t="str">
         <v>AS OF 11/23/2025</v>
       </c>
@@ -5514,18 +3572,6 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B70">
-        <v>-38.93</v>
-      </c>
-      <c r="C70" t="str">
-        <v>NENE CHICKEN SUNSHINE SUNSHINE</v>
-      </c>
-      <c r="D70" t="str">
-        <v/>
-      </c>
       <c r="F70" t="str">
         <v>macqbill owes tony 2.5</v>
       </c>
@@ -5547,18 +3593,6 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B71">
-        <v>-26.83</v>
-      </c>
-      <c r="C71" t="str">
-        <v>SQ *INDUS SPECIALTY CO St Kilda</v>
-      </c>
-      <c r="D71" t="str">
-        <v/>
-      </c>
       <c r="F71" t="str">
         <v>macqbill owes tony 2.3</v>
       </c>
@@ -5577,18 +3611,6 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B72">
-        <v>-15.23</v>
-      </c>
-      <c r="C72" t="str">
-        <v>KOMIKO.APP SAN FRANCISCO USA</v>
-      </c>
-      <c r="D72" t="str">
-        <v/>
-      </c>
       <c r="F72" s="2" t="str">
         <v>Macbill owes tony $1178</v>
       </c>
@@ -5607,18 +3629,6 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B73">
-        <v>-52.99</v>
-      </c>
-      <c r="C73" t="str">
-        <v>SQ *FOOD &amp; WINE EXPO Williamstown AUS</v>
-      </c>
-      <c r="D73" t="str">
-        <v/>
-      </c>
       <c r="F73" s="2" t="str">
         <v>Nugs owe macbill $561</v>
       </c>
@@ -5631,18 +3641,6 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B74">
-        <v>-22.22</v>
-      </c>
-      <c r="C74" t="str">
-        <v>SECURE PARKING THE STR MELBOURNE</v>
-      </c>
-      <c r="D74" t="str">
-        <v/>
-      </c>
       <c r="Q74">
         <v>-28.55</v>
       </c>
@@ -5652,18 +3650,6 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B75">
-        <v>-37.9</v>
-      </c>
-      <c r="C75" t="str">
-        <v>LS *BellPizza Mount Waverle AUS</v>
-      </c>
-      <c r="D75" t="str">
-        <v/>
-      </c>
       <c r="F75" t="str">
         <v>Nugs owe macbill $311 as of 22/01/2025</v>
       </c>
@@ -5680,18 +3666,6 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1">
-        <v>46102.458333333336</v>
-      </c>
-      <c r="B76">
-        <v>-18.89</v>
-      </c>
-      <c r="C76" t="str">
-        <v>PAYPAL *LEMONSQUEEZ 4029357733</v>
-      </c>
-      <c r="D76" t="str">
-        <v/>
-      </c>
       <c r="F76" t="str">
         <v xml:space="preserve">Jan bill &gt; Nugs to add 155.5 to "Japan" </v>
       </c>
@@ -5707,18 +3681,6 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1">
-        <v>46101.458333333336</v>
-      </c>
-      <c r="B77">
-        <v>-44</v>
-      </c>
-      <c r="C77" t="str">
-        <v>POP MART OCEANIA PTY L MELBOURNE</v>
-      </c>
-      <c r="D77" t="str">
-        <v/>
-      </c>
       <c r="F77" t="str">
         <v xml:space="preserve">Feb bill &gt; Nugs to add 155.5 to "Japan" </v>
       </c>
@@ -5734,18 +3696,6 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1">
-        <v>46101.458333333336</v>
-      </c>
-      <c r="B78">
-        <v>-9.6</v>
-      </c>
-      <c r="C78" t="str">
-        <v>WOOLWORTHS 3079 MARIBYRNONG</v>
-      </c>
-      <c r="D78" t="str">
-        <v/>
-      </c>
       <c r="Q78">
         <v>-1.03</v>
       </c>
@@ -5755,18 +3705,6 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1">
-        <v>46101.458333333336</v>
-      </c>
-      <c r="B79">
-        <v>-41.99</v>
-      </c>
-      <c r="C79" t="str">
-        <v>SQ *JASPER HIGHPOINT Maribyrnong</v>
-      </c>
-      <c r="D79" t="str">
-        <v/>
-      </c>
       <c r="Q79">
         <v>-0.49</v>
       </c>
@@ -5776,18 +3714,6 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1">
-        <v>46101.458333333336</v>
-      </c>
-      <c r="B80">
-        <v>-45.27</v>
-      </c>
-      <c r="C80" t="str">
-        <v>DUMPLING PLUS MARIBYRNONG</v>
-      </c>
-      <c r="D80" t="str">
-        <v/>
-      </c>
       <c r="Q80">
         <v>-37.5</v>
       </c>
@@ -5797,18 +3723,6 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1">
-        <v>46101.458333333336</v>
-      </c>
-      <c r="B81">
-        <v>-38</v>
-      </c>
-      <c r="C81" t="str">
-        <v>HARVEY NORMAN AV/IT MARIBYRNONG</v>
-      </c>
-      <c r="D81" t="str">
-        <v/>
-      </c>
       <c r="Q81">
         <v>-16.82</v>
       </c>
@@ -5818,18 +3732,6 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1">
-        <v>46101.458333333336</v>
-      </c>
-      <c r="B82">
-        <v>-30.98</v>
-      </c>
-      <c r="C82" t="str">
-        <v>PLINE PH HIGHPOINT MARIBYRNONG</v>
-      </c>
-      <c r="D82" t="str">
-        <v/>
-      </c>
       <c r="Q82">
         <v>-99.2</v>
       </c>
@@ -5839,18 +3741,6 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1">
-        <v>46100.458333333336</v>
-      </c>
-      <c r="B83">
-        <v>-42.65</v>
-      </c>
-      <c r="C83" t="str">
-        <v>McDonalds 950055 SUNSHINE</v>
-      </c>
-      <c r="D83" t="str">
-        <v/>
-      </c>
       <c r="Q83">
         <v>-66</v>
       </c>
@@ -5859,92 +3749,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="1">
-        <v>46098.458333333336</v>
-      </c>
-      <c r="B84">
-        <v>-631.43</v>
-      </c>
-      <c r="C84" t="str">
-        <v>GWW SUNBURY</v>
-      </c>
-      <c r="D84" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="1">
-        <v>46097.458333333336</v>
-      </c>
-      <c r="B85">
-        <v>-17.8</v>
-      </c>
-      <c r="C85" t="str">
-        <v>COLES 7795 BRAYBROOK</v>
-      </c>
-      <c r="D85" t="str">
-        <v/>
-      </c>
-    </row>
     <row r="86">
-      <c r="A86" s="1">
-        <v>46097.458333333336</v>
-      </c>
-      <c r="B86">
-        <v>-4.99</v>
-      </c>
-      <c r="C86" t="str">
-        <v>CENTRAL WEST ASIAN FOO BRAYBROOK</v>
-      </c>
-      <c r="D86" t="str">
-        <v/>
-      </c>
       <c r="F86">
         <v>1090</v>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="1">
-        <v>46097.458333333336</v>
-      </c>
-      <c r="B87">
-        <v>-21.14</v>
-      </c>
-      <c r="C87" t="str">
-        <v>KFL SUPERMARKET BRAYBR BRAYBROOK</v>
-      </c>
-      <c r="D87" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="1">
-        <v>46097.458333333336</v>
-      </c>
-      <c r="B88">
-        <v>-65</v>
-      </c>
-      <c r="C88" t="str">
-        <v>Superloop Limited BRISBANE</v>
-      </c>
-      <c r="D88" t="str">
-        <v/>
-      </c>
-    </row>
     <row r="89">
-      <c r="A89" s="1">
-        <v>46097.458333333336</v>
-      </c>
-      <c r="B89">
-        <v>-7.92</v>
-      </c>
-      <c r="C89" t="str">
-        <v>S &amp; S PRODUCE PTY LT BRAYBROOK</v>
-      </c>
-      <c r="D89" t="str">
-        <v/>
-      </c>
       <c r="G89">
         <v>399.96</v>
       </c>
@@ -5960,18 +3770,6 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1">
-        <v>46097.458333333336</v>
-      </c>
-      <c r="B90">
-        <v>-8.61</v>
-      </c>
-      <c r="C90" t="str">
-        <v>ALDI STORES WEST FOOTSCRA AUS</v>
-      </c>
-      <c r="D90" t="str">
-        <v/>
-      </c>
       <c r="G90">
         <v>199.98</v>
       </c>
@@ -5983,120 +3781,12 @@
         <v>66.66</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="1">
-        <v>46096.458333333336</v>
-      </c>
-      <c r="B91">
-        <v>-39.9</v>
-      </c>
-      <c r="C91" t="str">
-        <v>COLES 7795 BRAYBROOK</v>
-      </c>
-      <c r="D91" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="1">
-        <v>46096.458333333336</v>
-      </c>
-      <c r="B92">
-        <v>-22.43</v>
-      </c>
-      <c r="C92" t="str">
-        <v>Pacific D.lit Taylors Hill AUS</v>
-      </c>
-      <c r="D92" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="1">
-        <v>46096.458333333336</v>
-      </c>
-      <c r="B93">
-        <v>-131.25</v>
-      </c>
-      <c r="C93" t="str">
-        <v>Supre Sydney</v>
-      </c>
-      <c r="D93" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="1">
-        <v>46096.458333333336</v>
-      </c>
-      <c r="B94">
-        <v>-49.95</v>
-      </c>
-      <c r="C94" t="str">
-        <v>UPDOC--L.UPDOC.CO/CP SURRY HILLS</v>
-      </c>
-      <c r="D94" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="1">
-        <v>46096.458333333336</v>
-      </c>
-      <c r="B95">
-        <v>-25.58</v>
-      </c>
-      <c r="C95" t="str">
-        <v>ALDI STORES WEST FOOTSCRA AUS</v>
-      </c>
-      <c r="D95" t="str">
-        <v>t</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="1">
-        <v>46095.458333333336</v>
-      </c>
-      <c r="B96">
-        <v>-9.9</v>
-      </c>
-      <c r="C96" t="str">
-        <v>KC CHA PTY LTD. CARLTON</v>
-      </c>
-      <c r="D96" t="str">
-        <v>n</v>
-      </c>
-    </row>
     <row r="97">
-      <c r="A97" s="1">
-        <v>46095.458333333336</v>
-      </c>
-      <c r="B97">
-        <v>-7.9</v>
-      </c>
-      <c r="C97" t="str">
-        <v>Krispy Kreme Highpoint Maribyrnong</v>
-      </c>
-      <c r="D97" t="str">
-        <v>macq</v>
-      </c>
       <c r="G97" s="2">
         <v>6253.47</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1">
-        <v>46094.458333333336</v>
-      </c>
-      <c r="B98">
-        <v>-19.81</v>
-      </c>
-      <c r="C98" t="str">
-        <v>SQ *OLD MAN PHO EMPORI Melbourne</v>
-      </c>
-      <c r="D98" t="str">
-        <v>t</v>
-      </c>
       <c r="G98" t="str">
         <v/>
       </c>
@@ -6106,18 +3796,6 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1">
-        <v>46094.458333333336</v>
-      </c>
-      <c r="B99">
-        <v>-9.38</v>
-      </c>
-      <c r="C99" t="str">
-        <v>CWH MELBOURNE CENTRAL MELBOURNE</v>
-      </c>
-      <c r="D99" t="str">
-        <v/>
-      </c>
       <c r="G99" s="3" t="str">
         <v>Havies Distributed</v>
       </c>
@@ -6127,38 +3805,12 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1">
-        <v>46093.458333333336</v>
-      </c>
-      <c r="B100">
-        <v>-47.45</v>
-      </c>
-      <c r="C100" t="str">
-        <v>COLES 7664 MARIBYRNONG</v>
-      </c>
-      <c r="D100" t="str">
-        <v/>
-      </c>
       <c r="G100" s="2">
         <v>371.18499999999983</v>
       </c>
       <c r="H100">
         <f>SUM(H98:H99)</f>
         <v>12540</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="1">
-        <v>46093.458333333336</v>
-      </c>
-      <c r="B101">
-        <v>-21.19</v>
-      </c>
-      <c r="C101" t="str">
-        <v>FOODLE ASIAN GROCERY A MARIBYRNONG</v>
-      </c>
-      <c r="D101" t="str">
-        <v/>
       </c>
     </row>
     <row r="102">

</xml_diff>